<commit_message>
Add GitHub Actions workflows for Selenium, Load, and Vulnerability test suites
</commit_message>
<xml_diff>
--- a/load-tests/load-test-reports.xlsx
+++ b/load-tests/load-test-reports.xlsx
@@ -55,7 +55,7 @@
     <t>Requests Per Second (RPS)</t>
   </si>
   <si>
-    <t>399.04 req/sec</t>
+    <t>427.76 req/sec</t>
   </si>
   <si>
     <t>Successful Requests (2xx)</t>
@@ -73,19 +73,19 @@
     <t>Average Latency (ms)</t>
   </si>
   <si>
-    <t>249 ms</t>
+    <t>233 ms</t>
   </si>
   <si>
     <t>Minimum Latency (ms)</t>
   </si>
   <si>
-    <t>206 ms</t>
+    <t>205 ms</t>
   </si>
   <si>
     <t>Maximum Latency (ms)</t>
   </si>
   <si>
-    <t>1005 ms</t>
+    <t>1201 ms</t>
   </si>
 </sst>
 </file>
@@ -601,7 +601,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="6">
-        <v>24031</v>
+        <v>25766</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -617,7 +617,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="6">
-        <v>24031</v>
+        <v>25766</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>